<commit_message>
Edit About page text to explain draft values
</commit_message>
<xml_diff>
--- a/InputData/elec/SCGF/Soft Cap Growth Fraction.xlsx
+++ b/InputData/elec/SCGF/Soft Cap Growth Fraction.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\elec\SCGF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\SCGF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55E73B66-0694-4AFF-BA47-4B9DE56637CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7333E925-A4DE-4A42-8AEA-9DBDEB1A9E26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{D718C537-5235-45E1-A117-07B097D2BDF0}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{D718C537-5235-45E1-A117-07B097D2BDF0}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -152,7 +152,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
     <t>Source:</t>
   </si>
@@ -251,6 +251,81 @@
   </si>
   <si>
     <t>SCGF Soft Cap Growth Fraction</t>
+  </si>
+  <si>
+    <t>Source: Derived from historical growth rates of annual US capacity additions by technology (EIA-860 generator data; anchors listed below). Values are provisional engineering estimates pending a scripted EIA-860 derivation (see build-cap-calibration project) — the classification logic below is the durable content; individual values may be revised.</t>
+  </si>
+  <si>
+    <t>Notes:</t>
+  </si>
+  <si>
+    <r>
+      <t>SCGF sets how fast each technology's annual build limit can grow: each year, the limit may exceed the largest annual addition yet demonstrated (or the seed value, CSCSCbPT, where no cohort has been built) by this fraction. It is therefore calibrated to the fastest </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF0B0B0B"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>sustained multi-year growth in annual additions</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0B0B0B"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> each technology class has demonstrated historically — not to single-year spikes, which the cohort mechanism accommodates directly, and not to installed-capacity growth rates, which understate additions growth for young technologies.</t>
+    </r>
+  </si>
+  <si>
+    <t>Three rules generate the values:</t>
+  </si>
+  <si>
+    <t>1. Where a technology has a clear US deployment history, use its demonstrated additions-growth episode:</t>
+  </si>
+  <si>
+    <t>Solar PV, 0.40 — US utility-scale annual additions grew roughly tenfold over 2010–2016 (~40–45%/yr sustained).</t>
+  </si>
+  <si>
+    <t>Onshore wind, 0.35 — annual additions grew from ~0.7 to ~10 GW/yr over 1999–2009 (~30–35%/yr sustained).</t>
+  </si>
+  <si>
+    <t>Natural gas CC and peakers, 0.35 — the 1998–2002 build boom grew annual gas additions roughly fivefold in four years (&gt;40%/yr); 0.35 is set conservatively below the episode.</t>
+  </si>
+  <si>
+    <t>Nuclear, coal, gas steam, 0.15 — the 1966–1975 nuclear and 1970s coal build-outs sustained roughly 15%/yr growth in annual additions; representative of large single-site thermal projects generally, so also applied to biomass, geothermal, municipal solid waste, and oil-fired types, whose thin modern records do not support a higher figure.</t>
+  </si>
+  <si>
+    <t>Hydro, 0.10 — site-limited; retained at the pre-revision value.</t>
+  </si>
+  <si>
+    <t>2. Where US history is thin, use the closest overseas or supply-chain analogue:</t>
+  </si>
+  <si>
+    <t>Offshore wind, 0.30 — European deployment sustained ~25–35%/yr growth in annual additions over 2010–2023.</t>
+  </si>
+  <si>
+    <t>Hydrogen CT and CC, 0.30 — manufactured on the same gas-turbine supply chain as the gas fleet; assigned the gas-turbine class value rounded down.</t>
+  </si>
+  <si>
+    <t>3. Where no deployment history exists anywhere, interpolate between the classes by manufacturing character:</t>
+  </si>
+  <si>
+    <t>SMR, 0.25 and solar thermal, 0.25 — between the megaproject class (0.15) and the factory-manufactured class (0.35): the factory-fabrication premise argues above nuclear's 0.15, licensing and first-of-kind risk argue below solar/wind.</t>
+  </si>
+  <si>
+    <t>CCS types, 0.15–0.20 — megaproject retrofits on established gas/coal supply chains; gas CCS at 0.20 (larger host fleet and simpler retrofits), biomass/lignite CCS at 0.15.</t>
+  </si>
+  <si>
+    <t>The general pattern — factory-manufactured technologies ~0.35–0.40, project-built technologies ~0.15, hybrids between — reflects that additions growth is limited by manufacturing and installation-labor scale-up for modular technologies, and by site development and EPC capability for megaprojects.</t>
+  </si>
+  <si>
+    <t>SCGF is a single national vector: growth capability is a property of a technology's (national) supply chain, not of any state, so state deployments use these same values unchanged. Regional differentiation belongs in the seed (CSCSCbPT) and hard cap (HCFoTC) inputs.</t>
   </si>
 </sst>
 </file>
@@ -260,7 +335,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -304,19 +379,26 @@
       <sz val="10"/>
       <name val="MS Sans Serif"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0B0B0B"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF0B0B0B"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -336,11 +418,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma 2" xfId="5" xr:uid="{68733429-A9FA-4187-B93D-3BEA15728D17}"/>
@@ -796,7 +877,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{667665C7-8A8E-46D9-B686-64BA7741F669}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="73.85546875" customWidth="1"/>
@@ -826,13 +907,103 @@
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="A7" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -865,7 +1036,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -873,7 +1044,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -881,7 +1052,7 @@
         <v>26</v>
       </c>
       <c r="B4">
-        <v>0.1</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -889,7 +1060,7 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -905,7 +1076,7 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>0.1</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -913,7 +1084,7 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -921,7 +1092,7 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -929,7 +1100,7 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -937,7 +1108,7 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -945,7 +1116,7 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -953,7 +1124,7 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>0.1</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -961,7 +1132,7 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -969,7 +1140,7 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -977,7 +1148,7 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -985,7 +1156,7 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -993,7 +1164,7 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -1001,7 +1172,7 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -1009,7 +1180,7 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -1017,7 +1188,7 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -1025,7 +1196,7 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -1033,7 +1204,7 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -1041,7 +1212,7 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -1049,7 +1220,7 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>